<commit_message>
:up: pdfs de inf e RL cadastrados e algumas questões respondidas
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F621"/>
+  <dimension ref="A1:F640"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.5703125" customWidth="1" style="1" min="3" max="3"/>
@@ -16601,6 +16601,500 @@
         <v>1</v>
       </c>
     </row>
+    <row r="622">
+      <c r="A622" t="n">
+        <v>635</v>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>28/03/2026 07:40</t>
+        </is>
+      </c>
+      <c r="C622" t="n">
+        <v>27</v>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>Expressões Problemáticas</t>
+        </is>
+      </c>
+      <c r="F622" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="n">
+        <v>636</v>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>28/03/2026 07:41</t>
+        </is>
+      </c>
+      <c r="C623" t="n">
+        <v>28</v>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>Expressões Problemáticas</t>
+        </is>
+      </c>
+      <c r="F623" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="n">
+        <v>637</v>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>28/03/2026 07:46</t>
+        </is>
+      </c>
+      <c r="C624" t="n">
+        <v>183</v>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>Parênteses</t>
+        </is>
+      </c>
+      <c r="F624" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="n">
+        <v>638</v>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>28/03/2026 07:52</t>
+        </is>
+      </c>
+      <c r="C625" t="n">
+        <v>2278</v>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>Proteção contra vírus</t>
+        </is>
+      </c>
+      <c r="F625" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="n">
+        <v>639</v>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>28/03/2026 07:53</t>
+        </is>
+      </c>
+      <c r="C626" t="n">
+        <v>2443</v>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>Windows 10</t>
+        </is>
+      </c>
+      <c r="F626" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="n">
+        <v>640</v>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>28/03/2026 07:54</t>
+        </is>
+      </c>
+      <c r="C627" t="n">
+        <v>2586</v>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>Lei nº 12.527-2011</t>
+        </is>
+      </c>
+      <c r="F627" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="n">
+        <v>641</v>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>28/03/2026 07:55</t>
+        </is>
+      </c>
+      <c r="C628" t="n">
+        <v>2412</v>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>MS-Office M365 (OneDrive, Sharepoint e Teams)</t>
+        </is>
+      </c>
+      <c r="F628" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="n">
+        <v>642</v>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>28/03/2026 07:56</t>
+        </is>
+      </c>
+      <c r="C629" t="n">
+        <v>2561</v>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="F629" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="n">
+        <v>643</v>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>28/03/2026 07:56</t>
+        </is>
+      </c>
+      <c r="C630" t="n">
+        <v>2461</v>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>Windows 11</t>
+        </is>
+      </c>
+      <c r="F630" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="n">
+        <v>644</v>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>28/03/2026 07:57</t>
+        </is>
+      </c>
+      <c r="C631" t="n">
+        <v>2582</v>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>Lei nº 12.527-2011</t>
+        </is>
+      </c>
+      <c r="F631" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="n">
+        <v>645</v>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>28/03/2026 08:34</t>
+        </is>
+      </c>
+      <c r="C632" t="n">
+        <v>2553</v>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="F632" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="n">
+        <v>646</v>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>28/03/2026 08:38</t>
+        </is>
+      </c>
+      <c r="C633" t="n">
+        <v>2427</v>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>Windows 10</t>
+        </is>
+      </c>
+      <c r="F633" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="n">
+        <v>647</v>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>28/03/2026 08:39</t>
+        </is>
+      </c>
+      <c r="C634" t="n">
+        <v>2572</v>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>Lei nº 12.527-2011</t>
+        </is>
+      </c>
+      <c r="F634" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="n">
+        <v>648</v>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>28/03/2026 08:40</t>
+        </is>
+      </c>
+      <c r="C635" t="n">
+        <v>2454</v>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>Windows 11</t>
+        </is>
+      </c>
+      <c r="F635" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="n">
+        <v>649</v>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>28/03/2026 08:41</t>
+        </is>
+      </c>
+      <c r="C636" t="n">
+        <v>2533</v>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="F636" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="n">
+        <v>650</v>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>28/03/2026 08:43</t>
+        </is>
+      </c>
+      <c r="C637" t="n">
+        <v>2538</v>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="F637" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="n">
+        <v>651</v>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>28/03/2026 08:43</t>
+        </is>
+      </c>
+      <c r="C638" t="n">
+        <v>2442</v>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>Windows 10</t>
+        </is>
+      </c>
+      <c r="F638" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="n">
+        <v>652</v>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>28/03/2026 08:44</t>
+        </is>
+      </c>
+      <c r="C639" t="n">
+        <v>2480</v>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>Dados</t>
+        </is>
+      </c>
+      <c r="F639" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="n">
+        <v>653</v>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>28/03/2026 19:02</t>
+        </is>
+      </c>
+      <c r="C640" t="n">
+        <v>2117</v>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>Probabilidade</t>
+        </is>
+      </c>
+      <c r="F640" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
:up: algumas questões respondidas de GC
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F700"/>
+  <dimension ref="A1:F705"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.5703125" customWidth="1" style="1" min="3" max="3"/>
@@ -18663,6 +18663,144 @@
         <v>1</v>
       </c>
     </row>
+    <row r="701">
+      <c r="A701" t="n">
+        <v>714</v>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>04/04/2026 06:51</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>2624</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>Gestão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="F701" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="n">
+        <v>715</v>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>04/04/2026 06:54</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>749</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>Gestão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="F702" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="n">
+        <v>716</v>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>04/04/2026 06:57</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>2621</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>Gestão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="F703" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="n">
+        <v>717</v>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>04/04/2026 06:59</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>2623</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>Gestão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="F704" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="n">
+        <v>718</v>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>04/04/2026 07:01</t>
+        </is>
+      </c>
+      <c r="C705" t="n">
+        <v>2773</v>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>Gestão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="F705" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
:up: algumas questões respondidas - GC
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F803"/>
+  <dimension ref="A1:F808"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.5703125" customWidth="1" style="1" min="3" max="3"/>
@@ -21357,6 +21357,142 @@
         <v>0</v>
       </c>
     </row>
+    <row r="804">
+      <c r="A804" t="n">
+        <v>817</v>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>09/04/2026 13:02</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>2607</t>
+        </is>
+      </c>
+      <c r="D804" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E804" t="inlineStr">
+        <is>
+          <t>Gestão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="F804" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="n">
+        <v>818</v>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>09/04/2026 13:04</t>
+        </is>
+      </c>
+      <c r="C805" t="n">
+        <v>3034</v>
+      </c>
+      <c r="D805" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E805" t="inlineStr">
+        <is>
+          <t>Gestão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="F805" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="n">
+        <v>819</v>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>09/04/2026 13:04</t>
+        </is>
+      </c>
+      <c r="C806" t="n">
+        <v>3033</v>
+      </c>
+      <c r="D806" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E806" t="inlineStr">
+        <is>
+          <t>Gestão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="F806" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="n">
+        <v>820</v>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>09/04/2026 13:06</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>2610</t>
+        </is>
+      </c>
+      <c r="D807" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E807" t="inlineStr">
+        <is>
+          <t>Gestão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="F807" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="n">
+        <v>821</v>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>09/04/2026 13:11</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>2615</t>
+        </is>
+      </c>
+      <c r="D808" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E808" t="inlineStr">
+        <is>
+          <t>Gestão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="F808" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
:up: algumas questões respondidas - CC - ACP
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F861"/>
+  <dimension ref="A1:F864"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.5703125" customWidth="1" style="1" min="3" max="3"/>
@@ -22879,6 +22879,86 @@
         <v>1</v>
       </c>
     </row>
+    <row r="862">
+      <c r="A862" t="n">
+        <v>875</v>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>14/04/2026 03:40</t>
+        </is>
+      </c>
+      <c r="C862" t="n">
+        <v>2870</v>
+      </c>
+      <c r="D862" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E862" t="inlineStr">
+        <is>
+          <t>Apuração Do Custo De Produção</t>
+        </is>
+      </c>
+      <c r="F862" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="n">
+        <v>876</v>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>14/04/2026 03:44</t>
+        </is>
+      </c>
+      <c r="C863" t="n">
+        <v>3007</v>
+      </c>
+      <c r="D863" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E863" t="inlineStr">
+        <is>
+          <t>Apuração Do Custo De Produção</t>
+        </is>
+      </c>
+      <c r="F863" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="n">
+        <v>877</v>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>14/04/2026 03:46</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>3203</t>
+        </is>
+      </c>
+      <c r="D864" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E864" t="inlineStr">
+        <is>
+          <t>Apuração Do Custo De Produção</t>
+        </is>
+      </c>
+      <c r="F864" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
:lady_beetle: problema de erro em filtros por case consertado
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F864"/>
+  <dimension ref="A1:F866"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.5703125" customWidth="1" style="1" min="3" max="3"/>
@@ -22959,6 +22959,58 @@
         <v>0</v>
       </c>
     </row>
+    <row r="865">
+      <c r="A865" t="n">
+        <v>878</v>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>14/04/2026 04:15</t>
+        </is>
+      </c>
+      <c r="C865" t="n">
+        <v>3007</v>
+      </c>
+      <c r="D865" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E865" t="inlineStr">
+        <is>
+          <t>Apuração Do Custo De Produção</t>
+        </is>
+      </c>
+      <c r="F865" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="n">
+        <v>879</v>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>14/04/2026 04:16</t>
+        </is>
+      </c>
+      <c r="C866" t="n">
+        <v>2870</v>
+      </c>
+      <c r="D866" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E866" t="inlineStr">
+        <is>
+          <t>Apuração Do Custo De Produção</t>
+        </is>
+      </c>
+      <c r="F866" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
:lady_beetle: problema com banco de para De de CC substituição total realizada
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F866"/>
+  <dimension ref="A1:F868"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.5703125" customWidth="1" style="1" min="3" max="3"/>
@@ -23011,6 +23011,58 @@
         <v>0</v>
       </c>
     </row>
+    <row r="867">
+      <c r="A867" t="n">
+        <v>880</v>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>14/04/2026 05:02</t>
+        </is>
+      </c>
+      <c r="C867" t="n">
+        <v>2827</v>
+      </c>
+      <c r="D867" t="inlineStr">
+        <is>
+          <t>Contabilidade de Custos</t>
+        </is>
+      </c>
+      <c r="E867" t="inlineStr">
+        <is>
+          <t>Custos Diretos E Indiretos</t>
+        </is>
+      </c>
+      <c r="F867" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="n">
+        <v>881</v>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>14/04/2026 05:28</t>
+        </is>
+      </c>
+      <c r="C868" t="n">
+        <v>2863</v>
+      </c>
+      <c r="D868" t="inlineStr">
+        <is>
+          <t>Contabilidade de Custos</t>
+        </is>
+      </c>
+      <c r="E868" t="inlineStr">
+        <is>
+          <t>Custos Diretos E Indiretos</t>
+        </is>
+      </c>
+      <c r="F868" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
:up: simulado respondido e algumas questões corrigidas
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F983"/>
+  <dimension ref="A1:F1083"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.5703125" customWidth="1" style="1" min="3" max="3"/>
@@ -26093,6 +26093,2634 @@
         <v>1</v>
       </c>
     </row>
+    <row r="984">
+      <c r="A984" t="n">
+        <v>997</v>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:38</t>
+        </is>
+      </c>
+      <c r="C984" t="n">
+        <v>3265</v>
+      </c>
+      <c r="D984" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E984" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="F984" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" t="n">
+        <v>998</v>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:38</t>
+        </is>
+      </c>
+      <c r="C985" t="n">
+        <v>3264</v>
+      </c>
+      <c r="D985" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E985" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="F985" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" t="n">
+        <v>999</v>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:39</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>2646</t>
+        </is>
+      </c>
+      <c r="D986" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E986" t="inlineStr">
+        <is>
+          <t>Gestão da Tecnologia</t>
+        </is>
+      </c>
+      <c r="F986" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:39</t>
+        </is>
+      </c>
+      <c r="C987" t="n">
+        <v>3311</v>
+      </c>
+      <c r="D987" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E987" t="inlineStr">
+        <is>
+          <t>Engenharia de Métodos e Processos</t>
+        </is>
+      </c>
+      <c r="F987" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" t="n">
+        <v>1001</v>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:42</t>
+        </is>
+      </c>
+      <c r="C988" t="n">
+        <v>2768</v>
+      </c>
+      <c r="D988" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E988" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="F988" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" t="n">
+        <v>1002</v>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:43</t>
+        </is>
+      </c>
+      <c r="C989" t="n">
+        <v>3261</v>
+      </c>
+      <c r="D989" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E989" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="F989" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" t="n">
+        <v>1003</v>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:45</t>
+        </is>
+      </c>
+      <c r="C990" t="n">
+        <v>3027</v>
+      </c>
+      <c r="D990" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E990" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="F990" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" t="n">
+        <v>1004</v>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:45</t>
+        </is>
+      </c>
+      <c r="C991" t="n">
+        <v>2753</v>
+      </c>
+      <c r="D991" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E991" t="inlineStr">
+        <is>
+          <t>Gestão da Produção e Operações</t>
+        </is>
+      </c>
+      <c r="F991" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" t="n">
+        <v>1005</v>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:46</t>
+        </is>
+      </c>
+      <c r="C992" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D992" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E992" t="inlineStr">
+        <is>
+          <t>Gestão da Produção e Operações</t>
+        </is>
+      </c>
+      <c r="F992" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" t="n">
+        <v>1006</v>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:47</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>3325</t>
+        </is>
+      </c>
+      <c r="D993" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E993" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="F993" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" t="n">
+        <v>1007</v>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:48</t>
+        </is>
+      </c>
+      <c r="C994" t="n">
+        <v>3324</v>
+      </c>
+      <c r="D994" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E994" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="F994" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" t="n">
+        <v>1008</v>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:48</t>
+        </is>
+      </c>
+      <c r="C995" t="n">
+        <v>3323</v>
+      </c>
+      <c r="D995" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E995" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="F995" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" t="n">
+        <v>1009</v>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:48</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>3322</t>
+        </is>
+      </c>
+      <c r="D996" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E996" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="F996" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" t="n">
+        <v>1010</v>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:49</t>
+        </is>
+      </c>
+      <c r="C997" t="n">
+        <v>3266</v>
+      </c>
+      <c r="D997" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E997" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="F997" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="n">
+        <v>1011</v>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:49</t>
+        </is>
+      </c>
+      <c r="C998" t="n">
+        <v>2744</v>
+      </c>
+      <c r="D998" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E998" t="inlineStr">
+        <is>
+          <t>Pesquisa Operacional</t>
+        </is>
+      </c>
+      <c r="F998" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="n">
+        <v>1012</v>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:50</t>
+        </is>
+      </c>
+      <c r="C999" t="n">
+        <v>3258</v>
+      </c>
+      <c r="D999" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E999" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="F999" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="n">
+        <v>1013</v>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:50</t>
+        </is>
+      </c>
+      <c r="C1000" t="n">
+        <v>3344</v>
+      </c>
+      <c r="D1000" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1000" t="inlineStr">
+        <is>
+          <t>Engenharia de Produto</t>
+        </is>
+      </c>
+      <c r="F1000" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="n">
+        <v>1014</v>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:52</t>
+        </is>
+      </c>
+      <c r="C1001" t="n">
+        <v>3021</v>
+      </c>
+      <c r="D1001" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1001" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="F1001" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="n">
+        <v>1015</v>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:52</t>
+        </is>
+      </c>
+      <c r="C1002" t="n">
+        <v>3002</v>
+      </c>
+      <c r="D1002" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1002" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="F1002" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="n">
+        <v>1016</v>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:53</t>
+        </is>
+      </c>
+      <c r="C1003" t="n">
+        <v>3350</v>
+      </c>
+      <c r="D1003" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1003" t="inlineStr">
+        <is>
+          <t>Engenharia Organizacional</t>
+        </is>
+      </c>
+      <c r="F1003" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="n">
+        <v>1017</v>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:53</t>
+        </is>
+      </c>
+      <c r="C1004" t="n">
+        <v>3338</v>
+      </c>
+      <c r="D1004" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1004" t="inlineStr">
+        <is>
+          <t>Engenharia de Produto</t>
+        </is>
+      </c>
+      <c r="F1004" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="n">
+        <v>1018</v>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:54</t>
+        </is>
+      </c>
+      <c r="C1005" t="n">
+        <v>2746</v>
+      </c>
+      <c r="D1005" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1005" t="inlineStr">
+        <is>
+          <t>Pesquisa Operacional</t>
+        </is>
+      </c>
+      <c r="F1005" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="n">
+        <v>1019</v>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:55</t>
+        </is>
+      </c>
+      <c r="C1006" t="n">
+        <v>3313</v>
+      </c>
+      <c r="D1006" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1006" t="inlineStr">
+        <is>
+          <t>Engenharia de Métodos e Processos</t>
+        </is>
+      </c>
+      <c r="F1006" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="n">
+        <v>1020</v>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:56</t>
+        </is>
+      </c>
+      <c r="C1007" t="n">
+        <v>2776</v>
+      </c>
+      <c r="D1007" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1007" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="F1007" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="n">
+        <v>1021</v>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:56</t>
+        </is>
+      </c>
+      <c r="C1008" t="n">
+        <v>2760</v>
+      </c>
+      <c r="D1008" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1008" t="inlineStr">
+        <is>
+          <t>Gestão da Produção e Operações</t>
+        </is>
+      </c>
+      <c r="F1008" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="n">
+        <v>1022</v>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:57</t>
+        </is>
+      </c>
+      <c r="C1009" t="n">
+        <v>3346</v>
+      </c>
+      <c r="D1009" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1009" t="inlineStr">
+        <is>
+          <t>Engenharia de Produto</t>
+        </is>
+      </c>
+      <c r="F1009" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="n">
+        <v>1023</v>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:57</t>
+        </is>
+      </c>
+      <c r="C1010" t="n">
+        <v>3370</v>
+      </c>
+      <c r="D1010" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1010" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="F1010" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="n">
+        <v>1024</v>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:58</t>
+        </is>
+      </c>
+      <c r="C1011" t="n">
+        <v>2721</v>
+      </c>
+      <c r="D1011" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1011" t="inlineStr">
+        <is>
+          <t>Gestão de Projetos</t>
+        </is>
+      </c>
+      <c r="F1011" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="n">
+        <v>1025</v>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>17/04/2026 02:59</t>
+        </is>
+      </c>
+      <c r="C1012" t="n">
+        <v>2732</v>
+      </c>
+      <c r="D1012" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1012" t="inlineStr">
+        <is>
+          <t>Logística</t>
+        </is>
+      </c>
+      <c r="F1012" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="n">
+        <v>1026</v>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:00</t>
+        </is>
+      </c>
+      <c r="C1013" t="n">
+        <v>3020</v>
+      </c>
+      <c r="D1013" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1013" t="inlineStr">
+        <is>
+          <t>Gestão da Cadeia de Suprimentos</t>
+        </is>
+      </c>
+      <c r="F1013" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="n">
+        <v>1027</v>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:00</t>
+        </is>
+      </c>
+      <c r="C1014" t="n">
+        <v>3006</v>
+      </c>
+      <c r="D1014" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1014" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="F1014" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="n">
+        <v>1028</v>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:00</t>
+        </is>
+      </c>
+      <c r="C1015" t="n">
+        <v>3360</v>
+      </c>
+      <c r="D1015" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1015" t="inlineStr">
+        <is>
+          <t>Gestão da Tecnologia</t>
+        </is>
+      </c>
+      <c r="F1015" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="n">
+        <v>1029</v>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:01</t>
+        </is>
+      </c>
+      <c r="C1016" t="n">
+        <v>3025</v>
+      </c>
+      <c r="D1016" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1016" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="F1016" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="n">
+        <v>1030</v>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:02</t>
+        </is>
+      </c>
+      <c r="C1017" t="n">
+        <v>649</v>
+      </c>
+      <c r="D1017" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1017" t="inlineStr">
+        <is>
+          <t>Engenharia de Produto</t>
+        </is>
+      </c>
+      <c r="F1017" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="n">
+        <v>1031</v>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:03</t>
+        </is>
+      </c>
+      <c r="C1018" t="n">
+        <v>3359</v>
+      </c>
+      <c r="D1018" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1018" t="inlineStr">
+        <is>
+          <t>Engenharia Organizacional</t>
+        </is>
+      </c>
+      <c r="F1018" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="n">
+        <v>1032</v>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:04</t>
+        </is>
+      </c>
+      <c r="C1019" t="n">
+        <v>2777</v>
+      </c>
+      <c r="D1019" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1019" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="F1019" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="n">
+        <v>1033</v>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:06</t>
+        </is>
+      </c>
+      <c r="C1020" t="n">
+        <v>2757</v>
+      </c>
+      <c r="D1020" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1020" t="inlineStr">
+        <is>
+          <t>Engenharia de Métodos e Processos</t>
+        </is>
+      </c>
+      <c r="F1020" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="n">
+        <v>1034</v>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:07</t>
+        </is>
+      </c>
+      <c r="C1021" t="n">
+        <v>454</v>
+      </c>
+      <c r="D1021" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1021" t="inlineStr">
+        <is>
+          <t>Previsão da Demanda</t>
+        </is>
+      </c>
+      <c r="F1021" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="n">
+        <v>1035</v>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:08</t>
+        </is>
+      </c>
+      <c r="C1022" t="n">
+        <v>2728</v>
+      </c>
+      <c r="D1022" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1022" t="inlineStr">
+        <is>
+          <t>Gestão da Cadeia de Suprimentos</t>
+        </is>
+      </c>
+      <c r="F1022" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="n">
+        <v>1036</v>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:08</t>
+        </is>
+      </c>
+      <c r="C1023" t="n">
+        <v>3368</v>
+      </c>
+      <c r="D1023" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1023" t="inlineStr">
+        <is>
+          <t>Gestão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="F1023" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="n">
+        <v>1037</v>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:09</t>
+        </is>
+      </c>
+      <c r="C1024" t="n">
+        <v>3310</v>
+      </c>
+      <c r="D1024" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1024" t="inlineStr">
+        <is>
+          <t>Gestão da Produção e Operações</t>
+        </is>
+      </c>
+      <c r="F1024" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="n">
+        <v>1038</v>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:10</t>
+        </is>
+      </c>
+      <c r="C1025" t="n">
+        <v>3026</v>
+      </c>
+      <c r="D1025" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1025" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="F1025" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="n">
+        <v>1039</v>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:10</t>
+        </is>
+      </c>
+      <c r="C1026" t="n">
+        <v>3357</v>
+      </c>
+      <c r="D1026" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1026" t="inlineStr">
+        <is>
+          <t>Engenharia Organizacional</t>
+        </is>
+      </c>
+      <c r="F1026" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="n">
+        <v>1040</v>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:12</t>
+        </is>
+      </c>
+      <c r="C1027" t="n">
+        <v>2731</v>
+      </c>
+      <c r="D1027" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1027" t="inlineStr">
+        <is>
+          <t>Logística</t>
+        </is>
+      </c>
+      <c r="F1027" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="n">
+        <v>1041</v>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:12</t>
+        </is>
+      </c>
+      <c r="C1028" t="n">
+        <v>3252</v>
+      </c>
+      <c r="D1028" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1028" t="inlineStr">
+        <is>
+          <t>Engenharia Organizacional</t>
+        </is>
+      </c>
+      <c r="F1028" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="n">
+        <v>1042</v>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:13</t>
+        </is>
+      </c>
+      <c r="C1029" t="n">
+        <v>3358</v>
+      </c>
+      <c r="D1029" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1029" t="inlineStr">
+        <is>
+          <t>Engenharia Organizacional</t>
+        </is>
+      </c>
+      <c r="F1029" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="n">
+        <v>1043</v>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:14</t>
+        </is>
+      </c>
+      <c r="C1030" t="inlineStr">
+        <is>
+          <t>2631</t>
+        </is>
+      </c>
+      <c r="D1030" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1030" t="inlineStr">
+        <is>
+          <t>Gestão da Tecnologia</t>
+        </is>
+      </c>
+      <c r="F1030" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="n">
+        <v>1044</v>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:15</t>
+        </is>
+      </c>
+      <c r="C1031" t="n">
+        <v>3267</v>
+      </c>
+      <c r="D1031" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1031" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="F1031" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="n">
+        <v>1045</v>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:15</t>
+        </is>
+      </c>
+      <c r="C1032" t="n">
+        <v>2769</v>
+      </c>
+      <c r="D1032" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1032" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="F1032" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="n">
+        <v>1046</v>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:19</t>
+        </is>
+      </c>
+      <c r="C1033" t="n">
+        <v>3335</v>
+      </c>
+      <c r="D1033" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1033" t="inlineStr">
+        <is>
+          <t>Gestão de Investimentos e Risco</t>
+        </is>
+      </c>
+      <c r="F1033" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="n">
+        <v>1047</v>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:20</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
+        <is>
+          <t>3334</t>
+        </is>
+      </c>
+      <c r="D1034" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1034" t="inlineStr">
+        <is>
+          <t>Gestão de Investimentos e Risco</t>
+        </is>
+      </c>
+      <c r="F1034" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="n">
+        <v>1048</v>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:21</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>3333</t>
+        </is>
+      </c>
+      <c r="D1035" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1035" t="inlineStr">
+        <is>
+          <t>Gestão de Investimentos e Risco</t>
+        </is>
+      </c>
+      <c r="F1035" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="n">
+        <v>1049</v>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:22</t>
+        </is>
+      </c>
+      <c r="C1036" t="n">
+        <v>3318</v>
+      </c>
+      <c r="D1036" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1036" t="inlineStr">
+        <is>
+          <t>Gestão de Projetos</t>
+        </is>
+      </c>
+      <c r="F1036" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="n">
+        <v>1050</v>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:25</t>
+        </is>
+      </c>
+      <c r="C1037" t="n">
+        <v>2751</v>
+      </c>
+      <c r="D1037" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1037" t="inlineStr">
+        <is>
+          <t>Localização Industrial</t>
+        </is>
+      </c>
+      <c r="F1037" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="n">
+        <v>1051</v>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:26</t>
+        </is>
+      </c>
+      <c r="C1038" t="n">
+        <v>3263</v>
+      </c>
+      <c r="D1038" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1038" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="F1038" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="n">
+        <v>1052</v>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:26</t>
+        </is>
+      </c>
+      <c r="C1039" t="n">
+        <v>3362</v>
+      </c>
+      <c r="D1039" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1039" t="inlineStr">
+        <is>
+          <t>Gestão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="F1039" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="n">
+        <v>1053</v>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:26</t>
+        </is>
+      </c>
+      <c r="C1040" t="n">
+        <v>3364</v>
+      </c>
+      <c r="D1040" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1040" t="inlineStr">
+        <is>
+          <t>Gestão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="F1040" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="n">
+        <v>1054</v>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:27</t>
+        </is>
+      </c>
+      <c r="C1041" t="n">
+        <v>3235</v>
+      </c>
+      <c r="D1041" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1041" t="inlineStr">
+        <is>
+          <t>Gestão da Tecnologia</t>
+        </is>
+      </c>
+      <c r="F1041" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="n">
+        <v>1055</v>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:28</t>
+        </is>
+      </c>
+      <c r="C1042" t="n">
+        <v>3019</v>
+      </c>
+      <c r="D1042" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1042" t="inlineStr">
+        <is>
+          <t>Engenharia Organizacional</t>
+        </is>
+      </c>
+      <c r="F1042" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="n">
+        <v>1056</v>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:40</t>
+        </is>
+      </c>
+      <c r="C1043" t="n">
+        <v>2766</v>
+      </c>
+      <c r="D1043" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1043" t="inlineStr">
+        <is>
+          <t>Gestão da Manutenção e Confiabilidade</t>
+        </is>
+      </c>
+      <c r="F1043" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="n">
+        <v>1057</v>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:41</t>
+        </is>
+      </c>
+      <c r="C1044" t="n">
+        <v>2748</v>
+      </c>
+      <c r="D1044" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1044" t="inlineStr">
+        <is>
+          <t>Pesquisa Operacional</t>
+        </is>
+      </c>
+      <c r="F1044" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="n">
+        <v>1058</v>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:41</t>
+        </is>
+      </c>
+      <c r="C1045" t="n">
+        <v>2781</v>
+      </c>
+      <c r="D1045" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1045" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="F1045" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="n">
+        <v>1059</v>
+      </c>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:42</t>
+        </is>
+      </c>
+      <c r="C1046" t="n">
+        <v>3234</v>
+      </c>
+      <c r="D1046" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1046" t="inlineStr">
+        <is>
+          <t>Engenharia de Produto</t>
+        </is>
+      </c>
+      <c r="F1046" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" t="n">
+        <v>1060</v>
+      </c>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:43</t>
+        </is>
+      </c>
+      <c r="C1047" t="n">
+        <v>3223</v>
+      </c>
+      <c r="D1047" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1047" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="F1047" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" t="n">
+        <v>1061</v>
+      </c>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:44</t>
+        </is>
+      </c>
+      <c r="C1048" t="n">
+        <v>3336</v>
+      </c>
+      <c r="D1048" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1048" t="inlineStr">
+        <is>
+          <t>Engenharia de Produto</t>
+        </is>
+      </c>
+      <c r="F1048" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" t="n">
+        <v>1062</v>
+      </c>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:47</t>
+        </is>
+      </c>
+      <c r="C1049" t="n">
+        <v>2884</v>
+      </c>
+      <c r="D1049" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E1049" t="inlineStr">
+        <is>
+          <t>Equivalentes de Produção</t>
+        </is>
+      </c>
+      <c r="F1049" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" t="n">
+        <v>1063</v>
+      </c>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:48</t>
+        </is>
+      </c>
+      <c r="C1050" t="n">
+        <v>2869</v>
+      </c>
+      <c r="D1050" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E1050" t="inlineStr">
+        <is>
+          <t>Custos Diretos E Indiretos</t>
+        </is>
+      </c>
+      <c r="F1050" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" t="n">
+        <v>1064</v>
+      </c>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:48</t>
+        </is>
+      </c>
+      <c r="C1051" t="inlineStr">
+        <is>
+          <t>3231</t>
+        </is>
+      </c>
+      <c r="D1051" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E1051" t="inlineStr">
+        <is>
+          <t>Aspectos Introdutórios</t>
+        </is>
+      </c>
+      <c r="F1051" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" t="n">
+        <v>1065</v>
+      </c>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:49</t>
+        </is>
+      </c>
+      <c r="C1052" t="n">
+        <v>2484</v>
+      </c>
+      <c r="D1052" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E1052" t="inlineStr">
+        <is>
+          <t>Dados</t>
+        </is>
+      </c>
+      <c r="F1052" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" t="n">
+        <v>1066</v>
+      </c>
+      <c r="B1053" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:50</t>
+        </is>
+      </c>
+      <c r="C1053" t="n">
+        <v>2267</v>
+      </c>
+      <c r="D1053" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E1053" t="inlineStr">
+        <is>
+          <t>Proteção contra vírus</t>
+        </is>
+      </c>
+      <c r="F1053" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" t="n">
+        <v>1067</v>
+      </c>
+      <c r="B1054" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:50</t>
+        </is>
+      </c>
+      <c r="C1054" t="n">
+        <v>2369</v>
+      </c>
+      <c r="D1054" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E1054" t="inlineStr">
+        <is>
+          <t>MS-Office M365 (Power Point)</t>
+        </is>
+      </c>
+      <c r="F1054" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" t="n">
+        <v>1068</v>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:52</t>
+        </is>
+      </c>
+      <c r="C1055" t="n">
+        <v>2544</v>
+      </c>
+      <c r="D1055" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E1055" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="F1055" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" t="n">
+        <v>1069</v>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:53</t>
+        </is>
+      </c>
+      <c r="C1056" t="n">
+        <v>2498</v>
+      </c>
+      <c r="D1056" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E1056" t="inlineStr">
+        <is>
+          <t>Lei nº 13.709-2018</t>
+        </is>
+      </c>
+      <c r="F1056" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" t="n">
+        <v>1070</v>
+      </c>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:58</t>
+        </is>
+      </c>
+      <c r="C1057" t="n">
+        <v>2734</v>
+      </c>
+      <c r="D1057" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E1057" t="inlineStr">
+        <is>
+          <t>Juros Compostos</t>
+        </is>
+      </c>
+      <c r="F1057" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" t="n">
+        <v>1071</v>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>17/04/2026 03:59</t>
+        </is>
+      </c>
+      <c r="C1058" t="n">
+        <v>2735</v>
+      </c>
+      <c r="D1058" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E1058" t="inlineStr">
+        <is>
+          <t>Taxas</t>
+        </is>
+      </c>
+      <c r="F1058" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" t="n">
+        <v>1072</v>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>17/04/2026 04:00</t>
+        </is>
+      </c>
+      <c r="C1059" t="n">
+        <v>3398</v>
+      </c>
+      <c r="D1059" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E1059" t="inlineStr">
+        <is>
+          <t>Semântica</t>
+        </is>
+      </c>
+      <c r="F1059" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" t="n">
+        <v>1073</v>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>17/04/2026 04:09</t>
+        </is>
+      </c>
+      <c r="C1060" t="inlineStr">
+        <is>
+          <t>3419</t>
+        </is>
+      </c>
+      <c r="D1060" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E1060" t="inlineStr">
+        <is>
+          <t>Verbos</t>
+        </is>
+      </c>
+      <c r="F1060" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" t="n">
+        <v>1074</v>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>17/04/2026 04:10</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
+        <is>
+          <t>3418</t>
+        </is>
+      </c>
+      <c r="D1061" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E1061" t="inlineStr">
+        <is>
+          <t>Mecanismos de Coesão Textual</t>
+        </is>
+      </c>
+      <c r="F1061" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" t="n">
+        <v>1075</v>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>17/04/2026 04:11</t>
+        </is>
+      </c>
+      <c r="C1062" t="n">
+        <v>3417</v>
+      </c>
+      <c r="D1062" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E1062" t="inlineStr">
+        <is>
+          <t>Compreensão e Interpretação de Textos</t>
+        </is>
+      </c>
+      <c r="F1062" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" t="n">
+        <v>1076</v>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>17/04/2026 04:12</t>
+        </is>
+      </c>
+      <c r="C1063" t="n">
+        <v>3416</v>
+      </c>
+      <c r="D1063" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E1063" t="inlineStr">
+        <is>
+          <t>Semântica</t>
+        </is>
+      </c>
+      <c r="F1063" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" t="n">
+        <v>1077</v>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>17/04/2026 04:14</t>
+        </is>
+      </c>
+      <c r="C1064" t="n">
+        <v>3415</v>
+      </c>
+      <c r="D1064" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E1064" t="inlineStr">
+        <is>
+          <t>Funções Sintáticas</t>
+        </is>
+      </c>
+      <c r="F1064" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" t="n">
+        <v>1078</v>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t>17/04/2026 04:16</t>
+        </is>
+      </c>
+      <c r="C1065" t="inlineStr">
+        <is>
+          <t>3413</t>
+        </is>
+      </c>
+      <c r="D1065" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E1065" t="inlineStr">
+        <is>
+          <t>Semântica</t>
+        </is>
+      </c>
+      <c r="F1065" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" t="n">
+        <v>1079</v>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t>17/04/2026 04:17</t>
+        </is>
+      </c>
+      <c r="C1066" t="n">
+        <v>3412</v>
+      </c>
+      <c r="D1066" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E1066" t="inlineStr">
+        <is>
+          <t>Compreensão e Interpretação de Textos</t>
+        </is>
+      </c>
+      <c r="F1066" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" t="n">
+        <v>1080</v>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>17/04/2026 04:19</t>
+        </is>
+      </c>
+      <c r="C1067" t="n">
+        <v>3411</v>
+      </c>
+      <c r="D1067" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E1067" t="inlineStr">
+        <is>
+          <t>Concordância Verbal e Nominal</t>
+        </is>
+      </c>
+      <c r="F1067" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" t="n">
+        <v>1081</v>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>17/04/2026 04:22</t>
+        </is>
+      </c>
+      <c r="C1068" t="n">
+        <v>3410</v>
+      </c>
+      <c r="D1068" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E1068" t="inlineStr">
+        <is>
+          <t>Pontuação</t>
+        </is>
+      </c>
+      <c r="F1068" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" t="n">
+        <v>1082</v>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>17/04/2026 04:29</t>
+        </is>
+      </c>
+      <c r="C1069" t="inlineStr">
+        <is>
+          <t>3435</t>
+        </is>
+      </c>
+      <c r="D1069" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E1069" t="inlineStr">
+        <is>
+          <t>Semântica</t>
+        </is>
+      </c>
+      <c r="F1069" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" t="n">
+        <v>1083</v>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>17/04/2026 04:32</t>
+        </is>
+      </c>
+      <c r="C1070" t="n">
+        <v>3434</v>
+      </c>
+      <c r="D1070" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E1070" t="inlineStr">
+        <is>
+          <t>Funções Sintáticas</t>
+        </is>
+      </c>
+      <c r="F1070" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" t="n">
+        <v>1084</v>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>17/04/2026 04:33</t>
+        </is>
+      </c>
+      <c r="C1071" t="n">
+        <v>3433</v>
+      </c>
+      <c r="D1071" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E1071" t="inlineStr">
+        <is>
+          <t>Compreensão e Interpretação de Textos</t>
+        </is>
+      </c>
+      <c r="F1071" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" t="n">
+        <v>1085</v>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>17/04/2026 04:33</t>
+        </is>
+      </c>
+      <c r="C1072" t="n">
+        <v>3432</v>
+      </c>
+      <c r="D1072" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E1072" t="inlineStr">
+        <is>
+          <t>Compreensão e Interpretação de Textos</t>
+        </is>
+      </c>
+      <c r="F1072" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" t="n">
+        <v>1086</v>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t>17/04/2026 04:36</t>
+        </is>
+      </c>
+      <c r="C1073" t="n">
+        <v>3431</v>
+      </c>
+      <c r="D1073" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E1073" t="inlineStr">
+        <is>
+          <t>Semântica</t>
+        </is>
+      </c>
+      <c r="F1073" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" t="n">
+        <v>1087</v>
+      </c>
+      <c r="B1074" t="inlineStr">
+        <is>
+          <t>17/04/2026 04:37</t>
+        </is>
+      </c>
+      <c r="C1074" t="inlineStr">
+        <is>
+          <t>3430</t>
+        </is>
+      </c>
+      <c r="D1074" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E1074" t="inlineStr">
+        <is>
+          <t>Morfologia</t>
+        </is>
+      </c>
+      <c r="F1074" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" t="n">
+        <v>1088</v>
+      </c>
+      <c r="B1075" t="inlineStr">
+        <is>
+          <t>17/04/2026 04:42</t>
+        </is>
+      </c>
+      <c r="C1075" t="inlineStr">
+        <is>
+          <t>3400</t>
+        </is>
+      </c>
+      <c r="D1075" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E1075" t="inlineStr">
+        <is>
+          <t>Verbos</t>
+        </is>
+      </c>
+      <c r="F1075" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" t="n">
+        <v>1089</v>
+      </c>
+      <c r="B1076" t="inlineStr">
+        <is>
+          <t>17/04/2026 04:43</t>
+        </is>
+      </c>
+      <c r="C1076" t="n">
+        <v>3392</v>
+      </c>
+      <c r="D1076" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E1076" t="inlineStr">
+        <is>
+          <t>Compreensão e Interpretação de Textos</t>
+        </is>
+      </c>
+      <c r="F1076" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" t="n">
+        <v>1090</v>
+      </c>
+      <c r="B1077" t="inlineStr">
+        <is>
+          <t>17/04/2026 04:44</t>
+        </is>
+      </c>
+      <c r="C1077" t="n">
+        <v>3391</v>
+      </c>
+      <c r="D1077" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E1077" t="inlineStr">
+        <is>
+          <t>Compreensão e Interpretação de Textos</t>
+        </is>
+      </c>
+      <c r="F1077" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" t="n">
+        <v>1091</v>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>17/04/2026 04:45</t>
+        </is>
+      </c>
+      <c r="C1078" t="n">
+        <v>3393</v>
+      </c>
+      <c r="D1078" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E1078" t="inlineStr">
+        <is>
+          <t>Compreensão e Interpretação de Textos</t>
+        </is>
+      </c>
+      <c r="F1078" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" t="n">
+        <v>1092</v>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>17/04/2026 04:55</t>
+        </is>
+      </c>
+      <c r="C1079" t="n">
+        <v>2077</v>
+      </c>
+      <c r="D1079" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="E1079" t="inlineStr">
+        <is>
+          <t>Probabilidade</t>
+        </is>
+      </c>
+      <c r="F1079" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" t="n">
+        <v>1093</v>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>17/04/2026 05:00</t>
+        </is>
+      </c>
+      <c r="C1080" t="n">
+        <v>3390</v>
+      </c>
+      <c r="D1080" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="E1080" t="inlineStr">
+        <is>
+          <t>Probabilidade</t>
+        </is>
+      </c>
+      <c r="F1080" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" t="n">
+        <v>1094</v>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>17/04/2026 05:02</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>3389</t>
+        </is>
+      </c>
+      <c r="D1081" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="E1081" t="inlineStr">
+        <is>
+          <t>Análise Combinatória</t>
+        </is>
+      </c>
+      <c r="F1081" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" t="n">
+        <v>1095</v>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>17/04/2026 05:09</t>
+        </is>
+      </c>
+      <c r="C1082" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D1082" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="E1082" t="inlineStr">
+        <is>
+          <t>Teoria dos Conjuntos</t>
+        </is>
+      </c>
+      <c r="F1082" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" t="n">
+        <v>1096</v>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>17/04/2026 05:10</t>
+        </is>
+      </c>
+      <c r="C1083" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D1083" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="E1083" t="inlineStr">
+        <is>
+          <t>Teoria dos Conjuntos</t>
+        </is>
+      </c>
+      <c r="F1083" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
:up: algumas questões respondidas - GT e cards enxugados pela IA
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1094"/>
+  <dimension ref="A1:F1100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.5703125" customWidth="1" style="1" min="3" max="3"/>
@@ -29009,6 +29009,168 @@
         <v>1</v>
       </c>
     </row>
+    <row r="1095">
+      <c r="A1095" t="n">
+        <v>1108</v>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>18/04/2026 06:01</t>
+        </is>
+      </c>
+      <c r="C1095" t="n">
+        <v>2663</v>
+      </c>
+      <c r="D1095" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1095" t="inlineStr">
+        <is>
+          <t>Gestão da Tecnologia</t>
+        </is>
+      </c>
+      <c r="F1095" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" t="n">
+        <v>1109</v>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>18/04/2026 06:07</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>2647</t>
+        </is>
+      </c>
+      <c r="D1096" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1096" t="inlineStr">
+        <is>
+          <t>Gestão da Tecnologia</t>
+        </is>
+      </c>
+      <c r="F1096" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" t="n">
+        <v>1110</v>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>18/04/2026 07:55</t>
+        </is>
+      </c>
+      <c r="C1097" t="n">
+        <v>3247</v>
+      </c>
+      <c r="D1097" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1097" t="inlineStr">
+        <is>
+          <t>Gestão da Tecnologia</t>
+        </is>
+      </c>
+      <c r="F1097" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" t="n">
+        <v>1111</v>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>18/04/2026 07:56</t>
+        </is>
+      </c>
+      <c r="C1098" t="n">
+        <v>2661</v>
+      </c>
+      <c r="D1098" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1098" t="inlineStr">
+        <is>
+          <t>Gestão da Tecnologia</t>
+        </is>
+      </c>
+      <c r="F1098" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" t="n">
+        <v>1112</v>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>18/04/2026 07:56</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>3043</t>
+        </is>
+      </c>
+      <c r="D1099" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1099" t="inlineStr">
+        <is>
+          <t>Gestão da Tecnologia</t>
+        </is>
+      </c>
+      <c r="F1099" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" t="n">
+        <v>1113</v>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>18/04/2026 08:08</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>2639</t>
+        </is>
+      </c>
+      <c r="D1100" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1100" t="inlineStr">
+        <is>
+          <t>Gestão da Tecnologia</t>
+        </is>
+      </c>
+      <c r="F1100" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
:up: algumas questões respondidas - MF
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1106"/>
+  <dimension ref="A1:F1108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.5703125" customWidth="1" style="1" min="3" max="3"/>
@@ -29331,6 +29331,58 @@
         <v>1</v>
       </c>
     </row>
+    <row r="1107">
+      <c r="A1107" t="n">
+        <v>1120</v>
+      </c>
+      <c r="B1107" t="inlineStr">
+        <is>
+          <t>18/04/2026 10:27</t>
+        </is>
+      </c>
+      <c r="C1107" t="n">
+        <v>3198</v>
+      </c>
+      <c r="D1107" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="E1107" t="inlineStr">
+        <is>
+          <t>Equivalências e Negações Lógicas</t>
+        </is>
+      </c>
+      <c r="F1107" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" t="n">
+        <v>1121</v>
+      </c>
+      <c r="B1108" t="inlineStr">
+        <is>
+          <t>18/04/2026 10:45</t>
+        </is>
+      </c>
+      <c r="C1108" t="n">
+        <v>1958</v>
+      </c>
+      <c r="D1108" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="E1108" t="inlineStr">
+        <is>
+          <t>Equivalências e Negações Lógicas</t>
+        </is>
+      </c>
+      <c r="F1108" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
:up: algumas questões respondidas - CC
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1108"/>
+  <dimension ref="A1:F1111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.5703125" customWidth="1" style="1" min="3" max="3"/>
@@ -29383,6 +29383,86 @@
         <v>0</v>
       </c>
     </row>
+    <row r="1109">
+      <c r="A1109" t="n">
+        <v>1122</v>
+      </c>
+      <c r="B1109" t="inlineStr">
+        <is>
+          <t>18/04/2026 12:10</t>
+        </is>
+      </c>
+      <c r="C1109" t="n">
+        <v>3098</v>
+      </c>
+      <c r="D1109" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E1109" t="inlineStr">
+        <is>
+          <t>Taxas</t>
+        </is>
+      </c>
+      <c r="F1109" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" t="n">
+        <v>1123</v>
+      </c>
+      <c r="B1110" t="inlineStr">
+        <is>
+          <t>18/04/2026 12:58</t>
+        </is>
+      </c>
+      <c r="C1110" t="n">
+        <v>2836</v>
+      </c>
+      <c r="D1110" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E1110" t="inlineStr">
+        <is>
+          <t>Custos Diretos E Indiretos</t>
+        </is>
+      </c>
+      <c r="F1110" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" t="n">
+        <v>1124</v>
+      </c>
+      <c r="B1111" t="inlineStr">
+        <is>
+          <t>18/04/2026 13:14</t>
+        </is>
+      </c>
+      <c r="C1111" t="inlineStr">
+        <is>
+          <t>2881</t>
+        </is>
+      </c>
+      <c r="D1111" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E1111" t="inlineStr">
+        <is>
+          <t>Equivalentes de Produção</t>
+        </is>
+      </c>
+      <c r="F1111" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
:up: algumas questões respondidas - Manuten
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1111"/>
+  <dimension ref="A1:F1125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.5703125" customWidth="1" style="1" min="3" max="3"/>
@@ -29463,6 +29463,370 @@
         <v>0</v>
       </c>
     </row>
+    <row r="1112">
+      <c r="A1112" t="n">
+        <v>1125</v>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>18/04/2026 15:23</t>
+        </is>
+      </c>
+      <c r="C1112" t="n">
+        <v>2546</v>
+      </c>
+      <c r="D1112" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E1112" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="F1112" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" t="n">
+        <v>1126</v>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>18/04/2026 15:26</t>
+        </is>
+      </c>
+      <c r="C1113" t="n">
+        <v>2541</v>
+      </c>
+      <c r="D1113" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E1113" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="F1113" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" t="n">
+        <v>1127</v>
+      </c>
+      <c r="B1114" t="inlineStr">
+        <is>
+          <t>18/04/2026 15:26</t>
+        </is>
+      </c>
+      <c r="C1114" t="n">
+        <v>2531</v>
+      </c>
+      <c r="D1114" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E1114" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="F1114" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" t="n">
+        <v>1128</v>
+      </c>
+      <c r="B1115" t="inlineStr">
+        <is>
+          <t>18/04/2026 15:28</t>
+        </is>
+      </c>
+      <c r="C1115" t="n">
+        <v>2540</v>
+      </c>
+      <c r="D1115" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E1115" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="F1115" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" t="n">
+        <v>1129</v>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>18/04/2026 15:33</t>
+        </is>
+      </c>
+      <c r="C1116" t="n">
+        <v>2537</v>
+      </c>
+      <c r="D1116" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E1116" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="F1116" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" t="n">
+        <v>1130</v>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>18/04/2026 15:36</t>
+        </is>
+      </c>
+      <c r="C1117" t="n">
+        <v>2528</v>
+      </c>
+      <c r="D1117" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E1117" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="F1117" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" t="n">
+        <v>1131</v>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>18/04/2026 15:54</t>
+        </is>
+      </c>
+      <c r="C1118" t="n">
+        <v>2542</v>
+      </c>
+      <c r="D1118" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E1118" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="F1118" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" t="n">
+        <v>1132</v>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>18/04/2026 15:57</t>
+        </is>
+      </c>
+      <c r="C1119" t="n">
+        <v>2558</v>
+      </c>
+      <c r="D1119" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E1119" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="F1119" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" t="n">
+        <v>1133</v>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>18/04/2026 16:01</t>
+        </is>
+      </c>
+      <c r="C1120" t="n">
+        <v>2521</v>
+      </c>
+      <c r="D1120" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E1120" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="F1120" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" t="n">
+        <v>1134</v>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>18/04/2026 16:11</t>
+        </is>
+      </c>
+      <c r="C1121" t="n">
+        <v>2525</v>
+      </c>
+      <c r="D1121" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="E1121" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="F1121" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" t="n">
+        <v>1135</v>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>18/04/2026 17:37</t>
+        </is>
+      </c>
+      <c r="C1122" t="n">
+        <v>1777</v>
+      </c>
+      <c r="D1122" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1122" t="inlineStr">
+        <is>
+          <t>Gestão da Manutenção e Confiabilidade</t>
+        </is>
+      </c>
+      <c r="F1122" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" t="n">
+        <v>1136</v>
+      </c>
+      <c r="B1123" t="inlineStr">
+        <is>
+          <t>18/04/2026 17:43</t>
+        </is>
+      </c>
+      <c r="C1123" t="n">
+        <v>541</v>
+      </c>
+      <c r="D1123" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1123" t="inlineStr">
+        <is>
+          <t>Gestão da Manutenção e Confiabilidade</t>
+        </is>
+      </c>
+      <c r="F1123" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="n">
+        <v>1137</v>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>18/04/2026 18:02</t>
+        </is>
+      </c>
+      <c r="C1124" t="n">
+        <v>1778</v>
+      </c>
+      <c r="D1124" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1124" t="inlineStr">
+        <is>
+          <t>Gestão da Manutenção e Confiabilidade</t>
+        </is>
+      </c>
+      <c r="F1124" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="n">
+        <v>1138</v>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>18/04/2026 18:20</t>
+        </is>
+      </c>
+      <c r="C1125" t="n">
+        <v>529</v>
+      </c>
+      <c r="D1125" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E1125" t="inlineStr">
+        <is>
+          <t>Gestão da Manutenção e Confiabilidade</t>
+        </is>
+      </c>
+      <c r="F1125" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
:up: algumas questões respondidas - RL
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1206"/>
+  <dimension ref="A1:F1216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.5703125" customWidth="1" style="1" min="3" max="3"/>
@@ -31955,6 +31955,268 @@
         <v>0</v>
       </c>
     </row>
+    <row r="1207">
+      <c r="A1207" t="n">
+        <v>1220</v>
+      </c>
+      <c r="B1207" t="inlineStr">
+        <is>
+          <t>20/04/2026 19:15</t>
+        </is>
+      </c>
+      <c r="C1207" t="n">
+        <v>2001</v>
+      </c>
+      <c r="D1207" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="E1207" t="inlineStr">
+        <is>
+          <t>Lógica de Argumentação</t>
+        </is>
+      </c>
+      <c r="F1207" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" t="n">
+        <v>1221</v>
+      </c>
+      <c r="B1208" t="inlineStr">
+        <is>
+          <t>20/04/2026 19:18</t>
+        </is>
+      </c>
+      <c r="C1208" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D1208" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="E1208" t="inlineStr">
+        <is>
+          <t>Teoria dos Conjuntos</t>
+        </is>
+      </c>
+      <c r="F1208" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" t="n">
+        <v>1222</v>
+      </c>
+      <c r="B1209" t="inlineStr">
+        <is>
+          <t>20/04/2026 19:18</t>
+        </is>
+      </c>
+      <c r="C1209" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D1209" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="E1209" t="inlineStr">
+        <is>
+          <t>Teoria dos Conjuntos</t>
+        </is>
+      </c>
+      <c r="F1209" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" t="n">
+        <v>1223</v>
+      </c>
+      <c r="B1210" t="inlineStr">
+        <is>
+          <t>20/04/2026 19:19</t>
+        </is>
+      </c>
+      <c r="C1210" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="D1210" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="E1210" t="inlineStr">
+        <is>
+          <t>Teoria dos Conjuntos</t>
+        </is>
+      </c>
+      <c r="F1210" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" t="n">
+        <v>1224</v>
+      </c>
+      <c r="B1211" t="inlineStr">
+        <is>
+          <t>20/04/2026 19:23</t>
+        </is>
+      </c>
+      <c r="C1211" t="n">
+        <v>3284</v>
+      </c>
+      <c r="D1211" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="E1211" t="inlineStr">
+        <is>
+          <t>Equivalências e Negações Lógicas</t>
+        </is>
+      </c>
+      <c r="F1211" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" t="n">
+        <v>1225</v>
+      </c>
+      <c r="B1212" t="inlineStr">
+        <is>
+          <t>20/04/2026 19:36</t>
+        </is>
+      </c>
+      <c r="C1212" t="n">
+        <v>3278</v>
+      </c>
+      <c r="D1212" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="E1212" t="inlineStr">
+        <is>
+          <t>Equivalências e Negações Lógicas</t>
+        </is>
+      </c>
+      <c r="F1212" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" t="n">
+        <v>1226</v>
+      </c>
+      <c r="B1213" t="inlineStr">
+        <is>
+          <t>20/04/2026 19:43</t>
+        </is>
+      </c>
+      <c r="C1213" t="n">
+        <v>3280</v>
+      </c>
+      <c r="D1213" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="E1213" t="inlineStr">
+        <is>
+          <t>Equivalências e Negações Lógicas</t>
+        </is>
+      </c>
+      <c r="F1213" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="n">
+        <v>1227</v>
+      </c>
+      <c r="B1214" t="inlineStr">
+        <is>
+          <t>20/04/2026 19:48</t>
+        </is>
+      </c>
+      <c r="C1214" t="n">
+        <v>2030</v>
+      </c>
+      <c r="D1214" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="E1214" t="inlineStr">
+        <is>
+          <t>Teoria dos Conjuntos</t>
+        </is>
+      </c>
+      <c r="F1214" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="n">
+        <v>1228</v>
+      </c>
+      <c r="B1215" t="inlineStr">
+        <is>
+          <t>20/04/2026 19:51</t>
+        </is>
+      </c>
+      <c r="C1215" t="n">
+        <v>1941</v>
+      </c>
+      <c r="D1215" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="E1215" t="inlineStr">
+        <is>
+          <t>Equivalências e Negações Lógicas</t>
+        </is>
+      </c>
+      <c r="F1215" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="n">
+        <v>1229</v>
+      </c>
+      <c r="B1216" t="inlineStr">
+        <is>
+          <t>20/04/2026 19:55</t>
+        </is>
+      </c>
+      <c r="C1216" t="n">
+        <v>1940</v>
+      </c>
+      <c r="D1216" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="E1216" t="inlineStr">
+        <is>
+          <t>Equivalências e Negações Lógicas</t>
+        </is>
+      </c>
+      <c r="F1216" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
:up: ultimo commit antes de mudar para a preparacao da transpetro
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F291"/>
+  <dimension ref="A1:F297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8028,6 +8028,162 @@
         <v>0</v>
       </c>
     </row>
+    <row r="292">
+      <c r="A292" t="n">
+        <v>291</v>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>03/09/2026 10:25</t>
+        </is>
+      </c>
+      <c r="C292" t="n">
+        <v>4395</v>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Sistemas Lineares</t>
+        </is>
+      </c>
+      <c r="F292" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="n">
+        <v>292</v>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>03/09/2026 10:26</t>
+        </is>
+      </c>
+      <c r="C293" t="n">
+        <v>4388</v>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Sistemas Lineares</t>
+        </is>
+      </c>
+      <c r="F293" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="n">
+        <v>293</v>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>03/09/2026 10:28</t>
+        </is>
+      </c>
+      <c r="C294" t="n">
+        <v>4396</v>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Sistemas Lineares</t>
+        </is>
+      </c>
+      <c r="F294" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="n">
+        <v>294</v>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>03/09/2026 10:30</t>
+        </is>
+      </c>
+      <c r="C295" t="n">
+        <v>4390</v>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Sistemas Lineares</t>
+        </is>
+      </c>
+      <c r="F295" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="n">
+        <v>295</v>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>03/09/2026 10:38</t>
+        </is>
+      </c>
+      <c r="C296" t="n">
+        <v>4373</v>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Sistemas Lineares</t>
+        </is>
+      </c>
+      <c r="F296" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="n">
+        <v>296</v>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>03/09/2026 13:57</t>
+        </is>
+      </c>
+      <c r="C297" t="n">
+        <v>4376</v>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Sistemas Lineares</t>
+        </is>
+      </c>
+      <c r="F297" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>